<commit_message>
cad: bitacora corregida, misma masa por pieza que la flotacion
Columna relleno_% y fraccion maciza por pieza (100 % cajas estancas, tapas con junta y
ganchos; 40 % riel, bandejas y bisel): nodo simple 1228 g impresos (antes 584 con un factor
unico de 0.45), boya simple 1943 g, LR1 44 g, modular D200 1229 g. Incluye la boya propia y
el separador; hardware del V2 y de la boya con precios en amarillo. costo.factor_relleno en
desuso.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Proyecto/MóduloMecánico/salida/simple/BITACORA.xlsx
+++ b/Proyecto/MóduloMecánico/salida/simple/BITACORA.xlsx
@@ -605,7 +605,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>LanternGuard, prototipo simple Ø200: masa impresa, horas y costo</t>
+          <t>LanternGuard, prototipo simple Ø200 (nodo V2 + boya): masa impresa, horas y costo</t>
         </is>
       </c>
       <c r="B1" s="11" t="n"/>
@@ -651,15 +651,15 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Factor de relleno (estimado)</t>
+          <t>Impresora g/h (estimado)</t>
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>0.45</v>
+        <v>15</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>costo.factor_relleno</t>
+          <t>costo.g_por_h</t>
         </is>
       </c>
       <c r="D4" s="11" t="n"/>
@@ -669,15 +669,15 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Impresora g/h (estimado)</t>
+          <t>Filamento soles/kg (estimado)</t>
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>15</v>
+        <v>90</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>costo.g_por_h</t>
+          <t>costo.filamento_soles_kg</t>
         </is>
       </c>
       <c r="D5" s="11" t="n"/>
@@ -685,19 +685,9 @@
       <c r="F5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Filamento soles/kg (estimado)</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>costo.filamento_soles_kg</t>
-        </is>
-      </c>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
       <c r="D6" s="11" t="n"/>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
@@ -757,15 +747,15 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$L:$L)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$N:$N)</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$N:$N)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$P:$P)</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$O:$O)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A10,PIEZAS!$Q:$Q)</f>
         <v/>
       </c>
       <c r="E10" s="11">
@@ -784,15 +774,15 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$L:$L)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$N:$N)</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$N:$N)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$P:$P)</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$O:$O)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A11,PIEZAS!$Q:$Q)</f>
         <v/>
       </c>
       <c r="E11" s="11">
@@ -807,19 +797,19 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$L:$L)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$N:$N)</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$N:$N)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$P:$P)</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$O:$O)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A12,PIEZAS!$Q:$Q)</f>
         <v/>
       </c>
       <c r="E12" s="11">
@@ -838,15 +828,15 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$L:$L)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$N:$N)</f>
         <v/>
       </c>
       <c r="C13" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$N:$N)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$P:$P)</f>
         <v/>
       </c>
       <c r="D13" s="11">
-        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$O:$O)</f>
+        <f>SUMIF(PIEZAS!$B:$B,$A13,PIEZAS!$Q:$Q)</f>
         <v/>
       </c>
       <c r="E13" s="11">
@@ -896,7 +886,7 @@
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Costo de hardware: llenar los precios amarillos de HARDWARE. La fila modular D200 es para comparar.</t>
+          <t>Masa por pieza = la misma del calculo de flotacion (piel + relleno de cada pieza). Llenar los precios amarillos de HARDWARE para el costo total. La fila modular D200 es para comparar.</t>
         </is>
       </c>
       <c r="B16" s="11" t="n"/>
@@ -916,12 +906,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -929,12 +919,14 @@
     <col width="31" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="37" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -990,30 +982,40 @@
       </c>
       <c r="K1" s="13" t="inlineStr">
         <is>
-          <t>masa por pieza g (estimado)</t>
+          <t>relleno_%</t>
         </is>
       </c>
       <c r="L1" s="13" t="inlineStr">
         <is>
+          <t>fraccion maciza (piel + relleno)</t>
+        </is>
+      </c>
+      <c r="M1" s="13" t="inlineStr">
+        <is>
+          <t>masa por pieza g (estimado o slicer)</t>
+        </is>
+      </c>
+      <c r="N1" s="13" t="inlineStr">
+        <is>
           <t>masa total g</t>
         </is>
       </c>
-      <c r="M1" s="13" t="inlineStr">
-        <is>
-          <t>horas por pieza (estimado)</t>
-        </is>
-      </c>
-      <c r="N1" s="13" t="inlineStr">
+      <c r="O1" s="13" t="inlineStr">
+        <is>
+          <t>horas por pieza (estimado o slicer)</t>
+        </is>
+      </c>
+      <c r="P1" s="13" t="inlineStr">
         <is>
           <t>horas total</t>
         </is>
       </c>
-      <c r="O1" s="13" t="inlineStr">
+      <c r="Q1" s="13" t="inlineStr">
         <is>
           <t>costo S/</t>
         </is>
       </c>
-      <c r="P1" s="13" t="inlineStr">
+      <c r="R1" s="13" t="inlineStr">
         <is>
           <t>fuente masa y horas</t>
         </is>
@@ -1022,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>M1_caja_cuerpo</t>
+          <t>M1s_caja_cuerpo</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
@@ -1032,27 +1034,27 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Caja, cuerpo</t>
+          <t>M1 caja baja con bolsillos</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>159.6</v>
+        <v>147</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="G2" s="11" t="n">
-        <v>50</v>
+        <v>102.5</v>
       </c>
       <c r="H2" s="11" t="n">
-        <v>214.82</v>
+        <v>349.39</v>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
@@ -1060,16 +1062,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K2" s="11">
-        <f>H2*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L2" s="11">
-        <f>K2*D2</f>
-        <v/>
+      <c r="K2" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M2" s="11">
-        <f>K2/RESUMEN!$B$5</f>
+        <f>H2*RESUMEN!$B$3*L2</f>
         <v/>
       </c>
       <c r="N2" s="11">
@@ -1077,10 +1079,18 @@
         <v/>
       </c>
       <c r="O2" s="11">
-        <f>L2/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P2" s="11" t="inlineStr">
+        <f>M2/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P2" s="11">
+        <f>O2*D2</f>
+        <v/>
+      </c>
+      <c r="Q2" s="11">
+        <f>N2/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R2" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1099,7 +1109,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>Caja, tapa con asa</t>
+          <t>M2 caja, tapa con asa</t>
         </is>
       </c>
       <c r="D3" s="11" t="n">
@@ -1109,13 +1119,13 @@
         <v>63</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>159.6</v>
+        <v>147</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>129.41</v>
+        <v>136</v>
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
@@ -1127,16 +1137,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K3" s="11">
-        <f>H3*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L3" s="11">
-        <f>K3*D3</f>
-        <v/>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M3" s="11">
-        <f>K3/RESUMEN!$B$5</f>
+        <f>H3*RESUMEN!$B$3*L3</f>
         <v/>
       </c>
       <c r="N3" s="11">
@@ -1144,10 +1154,18 @@
         <v/>
       </c>
       <c r="O3" s="11">
-        <f>L3/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P3" s="11" t="inlineStr">
+        <f>M3/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P3" s="11">
+        <f>O3*D3</f>
+        <v/>
+      </c>
+      <c r="Q3" s="11">
+        <f>N3/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R3" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1156,7 +1174,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>M11_bandeja</t>
+          <t>M3s_riel_gancho</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -1166,44 +1184,44 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Bandeja</t>
+          <t>M3s riel con gancho, mitad</t>
         </is>
       </c>
       <c r="D4" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>127.6</v>
+        <v>141.5</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>94</v>
+        <v>77.2</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>35.64</v>
+        <v>85.28</v>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X+90</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K4" s="11">
-        <f>H4*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L4" s="11">
-        <f>K4*D4</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>riel 40 %, gancho 100 %</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>0.824</v>
       </c>
       <c r="M4" s="11">
-        <f>K4/RESUMEN!$B$5</f>
+        <f>H4*RESUMEN!$B$3*L4</f>
         <v/>
       </c>
       <c r="N4" s="11">
@@ -1211,10 +1229,18 @@
         <v/>
       </c>
       <c r="O4" s="11">
-        <f>L4/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P4" s="11" t="inlineStr">
+        <f>M4/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P4" s="11">
+        <f>O4*D4</f>
+        <v/>
+      </c>
+      <c r="Q4" s="11">
+        <f>N4/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R4" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1223,7 +1249,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>M3s_riel_mitad</t>
+          <t>M3t_tapa_bolsillo</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -1233,23 +1259,23 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Riel, mitad</t>
+          <t>M3t tapa del bolsillo</t>
         </is>
       </c>
       <c r="D5" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>215</v>
+        <v>117</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>57.3</v>
+        <v>3</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>148.45</v>
+        <v>11.14</v>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
@@ -1258,19 +1284,19 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K5" s="11">
-        <f>H5*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L5" s="11">
-        <f>K5*D5</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M5" s="11">
-        <f>K5/RESUMEN!$B$5</f>
+        <f>H5*RESUMEN!$B$3*L5</f>
         <v/>
       </c>
       <c r="N5" s="11">
@@ -1278,10 +1304,18 @@
         <v/>
       </c>
       <c r="O5" s="11">
-        <f>L5/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P5" s="11" t="inlineStr">
+        <f>M5/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P5" s="11">
+        <f>O5*D5</f>
+        <v/>
+      </c>
+      <c r="Q5" s="11">
+        <f>N5/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R5" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1290,7 +1324,7 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>M3t_tapa_bolsillo</t>
+          <t>M5s_capsula_tapa_pie</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -1300,44 +1334,44 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Tapa del bolsillo del lastre</t>
+          <t>M5s tapa con pie</t>
         </is>
       </c>
       <c r="D6" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>107</v>
+        <v>59.2</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>3</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>9.58</v>
+        <v>76.04000000000001</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K6" s="11">
-        <f>H6*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L6" s="11">
-        <f>K6*D6</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M6" s="11">
-        <f>K6/RESUMEN!$B$5</f>
+        <f>H6*RESUMEN!$B$3*L6</f>
         <v/>
       </c>
       <c r="N6" s="11">
@@ -1345,10 +1379,18 @@
         <v/>
       </c>
       <c r="O6" s="11">
-        <f>L6/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P6" s="11" t="inlineStr">
+        <f>M6/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P6" s="11">
+        <f>O6*D6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="11">
+        <f>N6/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R6" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1357,7 +1399,7 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>M5s_capsula_tapa_pie</t>
+          <t>M11_bandeja</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -1367,44 +1409,44 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Capsula, tapa con pie</t>
+          <t>M11 bandeja (M11_bandeja)</t>
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>96.8</v>
+        <v>115</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>64</v>
+        <v>114</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>95.90000000000001</v>
+        <v>30</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>94.26000000000001</v>
+        <v>39.91</v>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K7" s="11">
-        <f>H7*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L7" s="11">
-        <f>K7*D7</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>0.909</v>
       </c>
       <c r="M7" s="11">
-        <f>K7/RESUMEN!$B$5</f>
+        <f>H7*RESUMEN!$B$3*L7</f>
         <v/>
       </c>
       <c r="N7" s="11">
@@ -1412,10 +1454,18 @@
         <v/>
       </c>
       <c r="O7" s="11">
-        <f>L7/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P7" s="11" t="inlineStr">
+        <f>M7/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P7" s="11">
+        <f>O7*D7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="11">
+        <f>N7/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R7" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1424,7 +1474,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>M9s_gancho</t>
+          <t>M11_bandeja_sup</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -1434,27 +1484,27 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Gancho en C</t>
+          <t>M11 bandeja (M11_bandeja_sup)</t>
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>47.2</v>
+        <v>114</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>21.04</v>
+        <v>38.06</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>X+90</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1462,16 +1512,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K8" s="11">
-        <f>H8*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L8" s="11">
-        <f>K8*D8</f>
-        <v/>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>0.91</v>
       </c>
       <c r="M8" s="11">
-        <f>K8/RESUMEN!$B$5</f>
+        <f>H8*RESUMEN!$B$3*L8</f>
         <v/>
       </c>
       <c r="N8" s="11">
@@ -1479,10 +1529,18 @@
         <v/>
       </c>
       <c r="O8" s="11">
-        <f>L8/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P8" s="11" t="inlineStr">
+        <f>M8/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P8" s="11">
+        <f>O8*D8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="11">
+        <f>N8/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R8" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1501,7 +1559,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Capsula, cuerpo</t>
+          <t>M4 capsula, cuerpo</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
@@ -1529,16 +1587,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K9" s="11">
-        <f>H9*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L9" s="11">
-        <f>K9*D9</f>
-        <v/>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M9" s="11">
-        <f>K9/RESUMEN!$B$5</f>
+        <f>H9*RESUMEN!$B$3*L9</f>
         <v/>
       </c>
       <c r="N9" s="11">
@@ -1546,10 +1604,18 @@
         <v/>
       </c>
       <c r="O9" s="11">
-        <f>L9/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P9" s="11" t="inlineStr">
+        <f>M9/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P9" s="11">
+        <f>O9*D9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="11">
+        <f>N9/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R9" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1568,7 +1634,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Bisel de la ventana</t>
+          <t>M6 bisel</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
@@ -1596,16 +1662,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K10" s="11">
-        <f>H10*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L10" s="11">
-        <f>K10*D10</f>
-        <v/>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M10" s="11">
-        <f>K10/RESUMEN!$B$5</f>
+        <f>H10*RESUMEN!$B$3*L10</f>
         <v/>
       </c>
       <c r="N10" s="11">
@@ -1613,10 +1679,18 @@
         <v/>
       </c>
       <c r="O10" s="11">
-        <f>L10/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P10" s="11" t="inlineStr">
+        <f>M10/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P10" s="11">
+        <f>O10*D10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="11">
+        <f>N10/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R10" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1635,7 +1709,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Separador LR1</t>
+          <t>LR1 separador</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
@@ -1663,16 +1737,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K11" s="11">
-        <f>H11*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L11" s="11">
-        <f>K11*D11</f>
-        <v/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>0.766</v>
       </c>
       <c r="M11" s="11">
-        <f>K11/RESUMEN!$B$5</f>
+        <f>H11*RESUMEN!$B$3*L11</f>
         <v/>
       </c>
       <c r="N11" s="11">
@@ -1680,10 +1754,18 @@
         <v/>
       </c>
       <c r="O11" s="11">
-        <f>L11/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P11" s="11" t="inlineStr">
+        <f>M11/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P11" s="11">
+        <f>O11*D11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="11">
+        <f>N11/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R11" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1692,37 +1774,37 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>B1_casco_central</t>
+          <t>B1s_casco</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>B1s casco</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>209</v>
+        <v>240</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>141</v>
+        <v>220</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>312.68</v>
+        <v>753.49</v>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -1730,16 +1812,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K12" s="11">
-        <f>H12*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L12" s="11">
-        <f>K12*D12</f>
-        <v/>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M12" s="11">
-        <f>K12/RESUMEN!$B$5</f>
+        <f>H12*RESUMEN!$B$3*L12</f>
         <v/>
       </c>
       <c r="N12" s="11">
@@ -1747,10 +1829,18 @@
         <v/>
       </c>
       <c r="O12" s="11">
-        <f>L12/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P12" s="11" t="inlineStr">
+        <f>M12/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P12" s="11">
+        <f>O12*D12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="11">
+        <f>N12/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1759,54 +1849,54 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>B1b_bandeja</t>
+          <t>B2s_tapa</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Bandeja</t>
+          <t>B2s tapa</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>85</v>
+        <v>220</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>3</v>
+        <v>240</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>31.5</v>
+        <v>260.46</v>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K13" s="11">
-        <f>H13*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L13" s="11">
-        <f>K13*D13</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M13" s="11">
-        <f>K13/RESUMEN!$B$5</f>
+        <f>H13*RESUMEN!$B$3*L13</f>
         <v/>
       </c>
       <c r="N13" s="11">
@@ -1814,10 +1904,18 @@
         <v/>
       </c>
       <c r="O13" s="11">
-        <f>L13/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P13" s="11" t="inlineStr">
+        <f>M13/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P13" s="11">
+        <f>O13*D13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="11">
+        <f>N13/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1826,37 +1924,37 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>B2_tapa</t>
+          <t>B1bs_bandeja</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Tapa</t>
+          <t>B1bs bandeja</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>117</v>
+        <v>186</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>112.51</v>
+        <v>112.95</v>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
@@ -1864,16 +1962,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K14" s="11">
-        <f>H14*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L14" s="11">
-        <f>K14*D14</f>
-        <v/>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>0.897</v>
       </c>
       <c r="M14" s="11">
-        <f>K14/RESUMEN!$B$5</f>
+        <f>H14*RESUMEN!$B$3*L14</f>
         <v/>
       </c>
       <c r="N14" s="11">
@@ -1881,10 +1979,18 @@
         <v/>
       </c>
       <c r="O14" s="11">
-        <f>L14/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P14" s="11" t="inlineStr">
+        <f>M14/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>O14*D14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="11">
+        <f>N14/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1893,17 +1999,17 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>B3_larguero_panel</t>
+          <t>B3s_larguero</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Larguero del panel</t>
+          <t>B3s larguero del panel</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
@@ -1913,13 +2019,13 @@
         <v>24</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>33.62</v>
+        <v>28.42</v>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
@@ -1931,16 +2037,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K15" s="11">
-        <f>H15*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L15" s="11">
-        <f>K15*D15</f>
-        <v/>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>0.714</v>
       </c>
       <c r="M15" s="11">
-        <f>K15/RESUMEN!$B$5</f>
+        <f>H15*RESUMEN!$B$3*L15</f>
         <v/>
       </c>
       <c r="N15" s="11">
@@ -1948,10 +2054,18 @@
         <v/>
       </c>
       <c r="O15" s="11">
-        <f>L15/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P15" s="11" t="inlineStr">
+        <f>M15/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P15" s="11">
+        <f>O15*D15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="11">
+        <f>N15/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R15" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -1960,54 +2074,54 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>B4_mastil_antena</t>
+          <t>B5s_flotador</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Mastil de la antena</t>
+          <t>B5s flotador de esquina</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>91.47</v>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Y+90</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="F16" s="11" t="n">
-        <v>123</v>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>144</v>
-      </c>
-      <c r="H16" s="11" t="n">
-        <v>29.13</v>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>sin girar</t>
-        </is>
-      </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K16" s="11">
-        <f>H16*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L16" s="11">
-        <f>K16*D16</f>
-        <v/>
-      </c>
       <c r="M16" s="11">
-        <f>K16/RESUMEN!$B$5</f>
+        <f>H16*RESUMEN!$B$3*L16</f>
         <v/>
       </c>
       <c r="N16" s="11">
@@ -2015,10 +2129,18 @@
         <v/>
       </c>
       <c r="O16" s="11">
-        <f>L16/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P16" s="11" t="inlineStr">
+        <f>M16/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P16" s="11">
+        <f>O16*D16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="11">
+        <f>N16/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R16" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2027,54 +2149,54 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>B5_flotador</t>
+          <t>B6s_ojal</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Flotador</t>
+          <t>B6s ojal de amarre</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>48.4</v>
+        <v>26</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>72.09</v>
+        <v>8.31</v>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K17" s="11">
-        <f>H17*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L17" s="11">
-        <f>K17*D17</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M17" s="11">
-        <f>K17/RESUMEN!$B$5</f>
+        <f>H17*RESUMEN!$B$3*L17</f>
         <v/>
       </c>
       <c r="N17" s="11">
@@ -2082,10 +2204,18 @@
         <v/>
       </c>
       <c r="O17" s="11">
-        <f>L17/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P17" s="11" t="inlineStr">
+        <f>M17/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P17" s="11">
+        <f>O17*D17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="11">
+        <f>N17/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R17" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2094,33 +2224,33 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>B5b_tapa_flotador</t>
+          <t>M1_caja_cuerpo</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>modular D200</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Tapa del flotador</t>
+          <t>Caja, cuerpo</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>150</v>
+        <v>159.6</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>1.6</v>
+        <v>50</v>
       </c>
       <c r="H18" s="11" t="n">
-        <v>21.39</v>
+        <v>214.82</v>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
@@ -2129,19 +2259,19 @@
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K18" s="11">
-        <f>H18*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L18" s="11">
-        <f>K18*D18</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M18" s="11">
-        <f>K18/RESUMEN!$B$5</f>
+        <f>H18*RESUMEN!$B$3*L18</f>
         <v/>
       </c>
       <c r="N18" s="11">
@@ -2149,10 +2279,18 @@
         <v/>
       </c>
       <c r="O18" s="11">
-        <f>L18/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P18" s="11" t="inlineStr">
+        <f>M18/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P18" s="11">
+        <f>O18*D18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="11">
+        <f>N18/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R18" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2161,54 +2299,54 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>B6_ojal_amarre</t>
+          <t>M2_caja_tapa</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>boya</t>
+          <t>modular D200</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Ojal de amarre</t>
+          <t>Caja, tapa con asa</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>6</v>
+        <v>159.6</v>
       </c>
       <c r="H19" s="11" t="n">
-        <v>5.78</v>
+        <v>129.41</v>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K19" s="11">
-        <f>H19*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L19" s="11">
-        <f>K19*D19</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M19" s="11">
-        <f>K19/RESUMEN!$B$5</f>
+        <f>H19*RESUMEN!$B$3*L19</f>
         <v/>
       </c>
       <c r="N19" s="11">
@@ -2216,10 +2354,18 @@
         <v/>
       </c>
       <c r="O19" s="11">
-        <f>L19/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P19" s="11" t="inlineStr">
+        <f>M19/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P19" s="11">
+        <f>O19*D19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="11">
+        <f>N19/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R19" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2228,7 +2374,7 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>M1_caja_cuerpo</t>
+          <t>M11_bandeja</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -2238,23 +2384,23 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Caja, cuerpo</t>
+          <t>Bandeja</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>159.6</v>
+        <v>127.6</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>126</v>
+        <v>94</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="H20" s="11" t="n">
-        <v>214.82</v>
+        <v>35.64</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -2263,19 +2409,19 @@
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K20" s="11">
-        <f>H20*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L20" s="11">
-        <f>K20*D20</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>0.912</v>
       </c>
       <c r="M20" s="11">
-        <f>K20/RESUMEN!$B$5</f>
+        <f>H20*RESUMEN!$B$3*L20</f>
         <v/>
       </c>
       <c r="N20" s="11">
@@ -2283,10 +2429,18 @@
         <v/>
       </c>
       <c r="O20" s="11">
-        <f>L20/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P20" s="11" t="inlineStr">
+        <f>M20/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P20" s="11">
+        <f>O20*D20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="11">
+        <f>N20/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2295,7 +2449,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>M2_caja_tapa</t>
+          <t>M3_riel_central</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -2305,23 +2459,23 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Caja, tapa con asa</t>
+          <t>Riel, tramo central</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>63</v>
+        <v>69.8</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>159.6</v>
+        <v>140</v>
       </c>
       <c r="H21" s="11" t="n">
-        <v>129.41</v>
+        <v>170.11</v>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
@@ -2333,16 +2487,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K21" s="11">
-        <f>H21*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L21" s="11">
-        <f>K21*D21</f>
-        <v/>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M21" s="11">
-        <f>K21/RESUMEN!$B$5</f>
+        <f>H21*RESUMEN!$B$3*L21</f>
         <v/>
       </c>
       <c r="N21" s="11">
@@ -2350,10 +2504,18 @@
         <v/>
       </c>
       <c r="O21" s="11">
-        <f>L21/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P21" s="11" t="inlineStr">
+        <f>M21/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P21" s="11">
+        <f>O21*D21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="11">
+        <f>N21/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2362,7 +2524,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>M11_bandeja</t>
+          <t>M3_riel_ext</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -2372,44 +2534,44 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Bandeja</t>
+          <t>Riel, extension</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>44.76</v>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Y+90</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>127.6</v>
-      </c>
-      <c r="F22" s="11" t="n">
-        <v>94</v>
-      </c>
-      <c r="G22" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="H22" s="11" t="n">
-        <v>35.64</v>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>sin girar</t>
-        </is>
-      </c>
-      <c r="J22" s="11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K22" s="11">
-        <f>H22*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L22" s="11">
-        <f>K22*D22</f>
-        <v/>
-      </c>
       <c r="M22" s="11">
-        <f>K22/RESUMEN!$B$5</f>
+        <f>H22*RESUMEN!$B$3*L22</f>
         <v/>
       </c>
       <c r="N22" s="11">
@@ -2417,10 +2579,18 @@
         <v/>
       </c>
       <c r="O22" s="11">
-        <f>L22/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P22" s="11" t="inlineStr">
+        <f>M22/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P22" s="11">
+        <f>O22*D22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="11">
+        <f>N22/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R22" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2429,7 +2599,7 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>M3_riel_central</t>
+          <t>M3_riel_punta</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -2439,23 +2609,23 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Riel, tramo central</t>
+          <t>Riel, punta</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>69.8</v>
+        <v>30</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>170.11</v>
+        <v>25.32</v>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
@@ -2467,16 +2637,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K23" s="11">
-        <f>H23*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L23" s="11">
-        <f>K23*D23</f>
-        <v/>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>0.8090000000000001</v>
       </c>
       <c r="M23" s="11">
-        <f>K23/RESUMEN!$B$5</f>
+        <f>H23*RESUMEN!$B$3*L23</f>
         <v/>
       </c>
       <c r="N23" s="11">
@@ -2484,10 +2654,18 @@
         <v/>
       </c>
       <c r="O23" s="11">
-        <f>L23/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P23" s="11" t="inlineStr">
+        <f>M23/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P23" s="11">
+        <f>O23*D23</f>
+        <v/>
+      </c>
+      <c r="Q23" s="11">
+        <f>N23/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2496,7 +2674,7 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>M3_riel_ext</t>
+          <t>M3_tapa_bolsillo</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -2506,44 +2684,44 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Riel, extension</t>
+          <t>Tapa del bolsillo</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E24" s="11" t="n">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>115</v>
+        <v>3</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>44.76</v>
+        <v>9.58</v>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K24" s="11">
-        <f>H24*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L24" s="11">
-        <f>K24*D24</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>0.953</v>
       </c>
       <c r="M24" s="11">
-        <f>K24/RESUMEN!$B$5</f>
+        <f>H24*RESUMEN!$B$3*L24</f>
         <v/>
       </c>
       <c r="N24" s="11">
@@ -2551,10 +2729,18 @@
         <v/>
       </c>
       <c r="O24" s="11">
-        <f>L24/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P24" s="11" t="inlineStr">
+        <f>M24/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P24" s="11">
+        <f>O24*D24</f>
+        <v/>
+      </c>
+      <c r="Q24" s="11">
+        <f>N24/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R24" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2563,7 +2749,7 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>M3_riel_punta</t>
+          <t>M4_capsula_cuerpo</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -2573,27 +2759,27 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Riel, punta</t>
+          <t>Capsula, cuerpo</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="11" t="n">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>25.32</v>
+        <v>45.95</v>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>Y-90</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr">
@@ -2601,16 +2787,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K25" s="11">
-        <f>H25*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L25" s="11">
-        <f>K25*D25</f>
-        <v/>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M25" s="11">
-        <f>K25/RESUMEN!$B$5</f>
+        <f>H25*RESUMEN!$B$3*L25</f>
         <v/>
       </c>
       <c r="N25" s="11">
@@ -2618,10 +2804,18 @@
         <v/>
       </c>
       <c r="O25" s="11">
-        <f>L25/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P25" s="11" t="inlineStr">
+        <f>M25/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P25" s="11">
+        <f>O25*D25</f>
+        <v/>
+      </c>
+      <c r="Q25" s="11">
+        <f>N25/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R25" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2630,7 +2824,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>M3_tapa_bolsillo</t>
+          <t>M5_capsula_tapa</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -2640,44 +2834,44 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Tapa del bolsillo</t>
+          <t>Capsula, tapa con bisagra</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E26" s="11" t="n">
-        <v>107</v>
+        <v>33</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>9.58</v>
+        <v>23.47</v>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>X-90</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K26" s="11">
-        <f>H26*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L26" s="11">
-        <f>K26*D26</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L26" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M26" s="11">
-        <f>K26/RESUMEN!$B$5</f>
+        <f>H26*RESUMEN!$B$3*L26</f>
         <v/>
       </c>
       <c r="N26" s="11">
@@ -2685,10 +2879,18 @@
         <v/>
       </c>
       <c r="O26" s="11">
-        <f>L26/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P26" s="11" t="inlineStr">
+        <f>M26/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P26" s="11">
+        <f>O26*D26</f>
+        <v/>
+      </c>
+      <c r="Q26" s="11">
+        <f>N26/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R26" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2697,7 +2899,7 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>M4_capsula_cuerpo</t>
+          <t>M6_capsula_bisel</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -2707,44 +2909,44 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Capsula, cuerpo</t>
+          <t>Bisel</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E27" s="11" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="G27" s="11" t="n">
-        <v>44</v>
+        <v>2.5</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>45.95</v>
+        <v>1.89</v>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>Y-90</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K27" s="11">
-        <f>H27*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L27" s="11">
-        <f>K27*D27</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M27" s="11">
-        <f>K27/RESUMEN!$B$5</f>
+        <f>H27*RESUMEN!$B$3*L27</f>
         <v/>
       </c>
       <c r="N27" s="11">
@@ -2752,10 +2954,18 @@
         <v/>
       </c>
       <c r="O27" s="11">
-        <f>L27/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P27" s="11" t="inlineStr">
+        <f>M27/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P27" s="11">
+        <f>O27*D27</f>
+        <v/>
+      </c>
+      <c r="Q27" s="11">
+        <f>N27/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R27" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2764,7 +2974,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>M5_capsula_tapa</t>
+          <t>M9_gancho</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -2774,27 +2984,27 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Capsula, tapa con bisagra</t>
+          <t>Gancho al aro</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H28" s="11" t="n">
-        <v>23.47</v>
+        <v>19.51</v>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>X-90</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
@@ -2802,16 +3012,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="K28" s="11">
-        <f>H28*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L28" s="11">
-        <f>K28*D28</f>
-        <v/>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="n">
+        <v>0.735</v>
       </c>
       <c r="M28" s="11">
-        <f>K28/RESUMEN!$B$5</f>
+        <f>H28*RESUMEN!$B$3*L28</f>
         <v/>
       </c>
       <c r="N28" s="11">
@@ -2819,10 +3029,18 @@
         <v/>
       </c>
       <c r="O28" s="11">
-        <f>L28/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P28" s="11" t="inlineStr">
+        <f>M28/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P28" s="11">
+        <f>O28*D28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="11">
+        <f>N28/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R28" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2831,7 +3049,7 @@
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>M6_capsula_bisel</t>
+          <t>M10_carro_capsula</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
@@ -2841,44 +3059,44 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Bisel</t>
+          <t>Carro</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>42</v>
+        <v>80.8</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>42</v>
+        <v>38.6</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>2.5</v>
+        <v>85</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>1.89</v>
+        <v>54.5</v>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>Y-90</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K29" s="11">
-        <f>H29*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L29" s="11">
-        <f>K29*D29</f>
-        <v/>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>0.71</v>
       </c>
       <c r="M29" s="11">
-        <f>K29/RESUMEN!$B$5</f>
+        <f>H29*RESUMEN!$B$3*L29</f>
         <v/>
       </c>
       <c r="N29" s="11">
@@ -2886,10 +3104,18 @@
         <v/>
       </c>
       <c r="O29" s="11">
-        <f>L29/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P29" s="11" t="inlineStr">
+        <f>M29/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P29" s="11">
+        <f>O29*D29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="11">
+        <f>N29/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R29" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2898,7 +3124,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>M9_gancho</t>
+          <t>M12_perilla</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -2908,44 +3134,44 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Gancho al aro</t>
+          <t>Perilla</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="F30" s="11" t="n">
         <v>30</v>
       </c>
       <c r="G30" s="11" t="n">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="H30" s="11" t="n">
-        <v>19.51</v>
+        <v>6.71</v>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K30" s="11">
-        <f>H30*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L30" s="11">
-        <f>K30*D30</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>0.695</v>
       </c>
       <c r="M30" s="11">
-        <f>K30/RESUMEN!$B$5</f>
+        <f>H30*RESUMEN!$B$3*L30</f>
         <v/>
       </c>
       <c r="N30" s="11">
@@ -2953,10 +3179,18 @@
         <v/>
       </c>
       <c r="O30" s="11">
-        <f>L30/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P30" s="11" t="inlineStr">
+        <f>M30/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P30" s="11">
+        <f>O30*D30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="11">
+        <f>N30/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R30" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -2965,7 +3199,7 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>M10_carro_capsula</t>
+          <t>M13_casquillo_D8</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -2975,44 +3209,44 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Carro</t>
+          <t>Casquillo Ø8</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E31" s="11" t="n">
-        <v>80.8</v>
+        <v>15.7</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>38.6</v>
+        <v>20</v>
       </c>
       <c r="G31" s="11" t="n">
-        <v>85</v>
+        <v>13.5</v>
       </c>
       <c r="H31" s="11" t="n">
-        <v>54.5</v>
+        <v>1.61</v>
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>Y-90</t>
+          <t>X-90</t>
         </is>
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K31" s="11">
-        <f>H31*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L31" s="11">
-        <f>K31*D31</f>
-        <v/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>0.972</v>
       </c>
       <c r="M31" s="11">
-        <f>K31/RESUMEN!$B$5</f>
+        <f>H31*RESUMEN!$B$3*L31</f>
         <v/>
       </c>
       <c r="N31" s="11">
@@ -3020,10 +3254,18 @@
         <v/>
       </c>
       <c r="O31" s="11">
-        <f>L31/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P31" s="11" t="inlineStr">
+        <f>M31/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P31" s="11">
+        <f>O31*D31</f>
+        <v/>
+      </c>
+      <c r="Q31" s="11">
+        <f>N31/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R31" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
@@ -3032,7 +3274,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>M12_perilla</t>
+          <t>M14_pestillo</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -3042,27 +3284,27 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Perilla</t>
+          <t>Pestillo</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E32" s="11" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>30</v>
+        <v>35.2</v>
       </c>
       <c r="G32" s="11" t="n">
-        <v>12</v>
+        <v>3.6</v>
       </c>
       <c r="H32" s="11" t="n">
-        <v>6.71</v>
+        <v>0.92</v>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>X+90</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
@@ -3070,16 +3312,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K32" s="11">
-        <f>H32*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L32" s="11">
-        <f>K32*D32</f>
-        <v/>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="M32" s="11">
-        <f>K32/RESUMEN!$B$5</f>
+        <f>H32*RESUMEN!$B$3*L32</f>
         <v/>
       </c>
       <c r="N32" s="11">
@@ -3087,188 +3329,66 @@
         <v/>
       </c>
       <c r="O32" s="11">
-        <f>L32/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P32" s="11" t="inlineStr">
+        <f>M32/RESUMEN!$B$4</f>
+        <v/>
+      </c>
+      <c r="P32" s="11">
+        <f>O32*D32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="11">
+        <f>N32/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R32" s="11" t="inlineStr">
         <is>
           <t>estimado</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>M13_casquillo_D8</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>modular D200</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>Casquillo Ø8</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" s="11" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="F33" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="H33" s="11" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="I33" s="11" t="inlineStr">
-        <is>
-          <t>X-90</t>
-        </is>
-      </c>
-      <c r="J33" s="11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K33" s="11">
-        <f>H33*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L33" s="11">
-        <f>K33*D33</f>
-        <v/>
-      </c>
-      <c r="M33" s="11">
-        <f>K33/RESUMEN!$B$5</f>
-        <v/>
-      </c>
-      <c r="N33" s="11">
-        <f>M33*D33</f>
-        <v/>
-      </c>
-      <c r="O33" s="11">
-        <f>L33/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P33" s="11" t="inlineStr">
-        <is>
-          <t>estimado</t>
-        </is>
-      </c>
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+      <c r="H33" s="11" t="n"/>
+      <c r="I33" s="11" t="n"/>
+      <c r="J33" s="11" t="n"/>
+      <c r="K33" s="11" t="n"/>
+      <c r="L33" s="11" t="n"/>
+      <c r="M33" s="11" t="n"/>
+      <c r="N33" s="11" t="n"/>
+      <c r="O33" s="11" t="n"/>
+      <c r="P33" s="11" t="n"/>
+      <c r="Q33" s="11" t="n"/>
+      <c r="R33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>M14_pestillo</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>modular D200</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>Pestillo</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="F34" s="11" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="G34" s="11" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="H34" s="11" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="I34" s="11" t="inlineStr">
-        <is>
-          <t>X+90</t>
-        </is>
-      </c>
-      <c r="J34" s="11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K34" s="11">
-        <f>H34*RESUMEN!$B$3*RESUMEN!$B$4</f>
-        <v/>
-      </c>
-      <c r="L34" s="11">
-        <f>K34*D34</f>
-        <v/>
-      </c>
-      <c r="M34" s="11">
-        <f>K34/RESUMEN!$B$5</f>
-        <v/>
-      </c>
-      <c r="N34" s="11">
-        <f>M34*D34</f>
-        <v/>
-      </c>
-      <c r="O34" s="11">
-        <f>L34/1000*RESUMEN!$B$6</f>
-        <v/>
-      </c>
-      <c r="P34" s="11" t="inlineStr">
-        <is>
-          <t>estimado</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="n"/>
-      <c r="G35" s="11" t="n"/>
-      <c r="H35" s="11" t="n"/>
-      <c r="I35" s="11" t="n"/>
-      <c r="J35" s="11" t="n"/>
-      <c r="K35" s="11" t="n"/>
-      <c r="L35" s="11" t="n"/>
-      <c r="M35" s="11" t="n"/>
-      <c r="N35" s="11" t="n"/>
-      <c r="O35" s="11" t="n"/>
-      <c r="P35" s="11" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>Soportes: si el voladizo en la orientacion de impresion pasa de 300 mm². Masa estimada = volumen x densidad x factor de relleno; horas = masa / g por hora (RESUMEN).</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="n"/>
-      <c r="C36" s="11" t="n"/>
-      <c r="D36" s="11" t="n"/>
-      <c r="E36" s="11" t="n"/>
-      <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="n"/>
-      <c r="H36" s="11" t="n"/>
-      <c r="I36" s="11" t="n"/>
-      <c r="J36" s="11" t="n"/>
-      <c r="K36" s="11" t="n"/>
-      <c r="L36" s="11" t="n"/>
-      <c r="M36" s="11" t="n"/>
-      <c r="N36" s="11" t="n"/>
-      <c r="O36" s="11" t="n"/>
-      <c r="P36" s="11" t="n"/>
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Soportes: voladizo en la orientacion de impresion &gt; 300 mm². Masa = volumen x densidad x fraccion maciza (piel de impresion.cascara + relleno); horas = masa / g por hora (RESUMEN).</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="11" t="n"/>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n"/>
+      <c r="L34" s="11" t="n"/>
+      <c r="M34" s="11" t="n"/>
+      <c r="N34" s="11" t="n"/>
+      <c r="O34" s="11" t="n"/>
+      <c r="P34" s="11" t="n"/>
+      <c r="Q34" s="11" t="n"/>
+      <c r="R34" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3281,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3341,7 +3461,7 @@
         </is>
       </c>
       <c r="D2" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2" s="12" t="n"/>
       <c r="F2" s="11">
@@ -3357,7 +3477,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 8 + inserto termico M3 (bandeja)</t>
+          <t>Tornillo M3 x 8 + inserto termico M3 (bandejas)</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -3407,16 +3527,16 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M4 x 12 + inserto termico M4 (riel a la caja)</t>
+          <t>Tornillo M2 autorroscante (bisel)</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2 x 6</t>
         </is>
       </c>
       <c r="D5" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="12" t="n"/>
       <c r="F5" s="11">
@@ -3432,16 +3552,16 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M2 autorroscante (bisel)</t>
+          <t>Cordon de junta torica Ø2 (caja + 2 capsulas, +10 %)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>M2 x 6</t>
+          <t>970 mm</t>
         </is>
       </c>
       <c r="D6" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E6" s="12" t="n"/>
       <c r="F6" s="11">
@@ -3457,16 +3577,16 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Cordon de junta torica Ø2 (caja + 2 capsulas, +10 %)</t>
+          <t>Prensaestopas PG7 con contratuerca (3 caja + 2 capsulas)</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>950 mm</t>
+          <t>PG7</t>
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E7" s="12" t="n"/>
       <c r="F7" s="11">
@@ -3482,16 +3602,16 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Prensaestopas PG7 con contratuerca (3 caja + 2 capsulas)</t>
+          <t>Disco de acrilico de la ventana</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PG7</t>
+          <t>Ø30 x 3</t>
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E8" s="12" t="n"/>
       <c r="F8" s="11">
@@ -3507,16 +3627,16 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Disco de acrilico de la ventana</t>
+          <t>Grillete o argolla de inox (izado)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Ø30 x 3</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="12" t="n"/>
       <c r="F9" s="11">
@@ -3530,18 +3650,18 @@
           <t>nodo simple</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Grillete o argolla de inox (izado)</t>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Tornillo M4 x 20 + inserto termico M4 (bridas del riel a la caja)</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E10" s="12" t="n"/>
       <c r="F10" s="11">
@@ -3557,7 +3677,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 20 + tuerca (union del riel)</t>
+          <t>Tornillo M3 x 8 avellanado + inserto M3 (tapas del bolsillo)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -3582,12 +3702,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 8 avellanado + inserto M3 (tapa del bolsillo)</t>
+          <t>Tornillo M4 x 45 + tuerca (pie de las capsulas)</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D12" s="11" t="n">
@@ -3607,16 +3727,16 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M4 x 12 + tuerca M4 en la ranura T (ganchos)</t>
+          <t>Correa textil</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>25 x 300 mm</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E13" s="12" t="n"/>
       <c r="F13" s="11">
@@ -3632,16 +3752,16 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M4 x 45 + tuerca (pie de las capsulas)</t>
+          <t>Pletina de inox</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>25 x 5 x 100</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E14" s="12" t="n"/>
       <c r="F14" s="11">
@@ -3652,21 +3772,21 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>nodo simple</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Correa textil</t>
+          <t>Tornillo M3 x 12 + inserto M3 (tapa de la boya)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>25 x 300 mm</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="11">
@@ -3677,21 +3797,21 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>nodo simple</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Pletina de inox</t>
+          <t>Tornillo M3 + inserto M3 (portabaterias y bandeja)</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>25 x 5 x 100</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E16" s="12" t="n"/>
       <c r="F16" s="11">
@@ -3702,12 +3822,12 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 12 + inserto termico M3 (tapa de la caja)</t>
+          <t>Tornillo M3 x 30 + inserto M3 (largueros a la tapa)</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -3716,7 +3836,7 @@
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E17" s="12" t="n"/>
       <c r="F17" s="11">
@@ -3727,12 +3847,12 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 8 + inserto termico M3 (bandeja)</t>
+          <t>Tornillo M3 + inserto M3 (panel a los largueros)</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -3752,17 +3872,17 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 16 + tuerca (capsulas)</t>
+          <t>Perno M5 x 120 inox + inserto M5 (flotadores)</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
@@ -3777,21 +3897,21 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M4 x 12 + inserto termico M4 (riel a la caja)</t>
+          <t>Tornillo M5 + inserto M5 (ojal de amarre)</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E20" s="12" t="n"/>
       <c r="F20" s="11">
@@ -3802,21 +3922,21 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M2 autorroscante (bisel)</t>
+          <t>Cordon de junta torica Ø2 (tapa de la boya, +10 %)</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>M2 x 6</t>
+          <t>900 mm</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E21" s="12" t="n"/>
       <c r="F21" s="11">
@@ -3827,21 +3947,21 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Cordon de junta torica Ø2 (caja + 2 capsulas, +10 %)</t>
+          <t>Prensaestopas PG7 (umbilical y panel)</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>950 mm</t>
+          <t>PG7</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="12" t="n"/>
       <c r="F22" s="11">
@@ -3852,21 +3972,21 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Prensaestopas PG7 con contratuerca (3 caja + 2 capsulas)</t>
+          <t>boya simple</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Tapon de la boca de llenado de los flotadores (o sello con PETG)</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>PG7</t>
+          <t>Ø10</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="11">
@@ -3877,21 +3997,21 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Disco de acrilico de la ventana</t>
+          <t>Manguera flexible U1 de referencia</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Ø30 x 3</t>
+          <t>Ø10</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="12" t="n"/>
       <c r="F24" s="11">
@@ -3902,17 +4022,17 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Grillete o argolla de inox (izado)</t>
+          <t>Cabo de amarre C1 boya-linterna</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>Ø4</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
@@ -3932,16 +4052,16 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Varilla roscada M8 (8.8)</t>
+          <t>Tornillo M3 x 12 + inserto termico M3 (tapa de la caja)</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>451 mm</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E26" s="12" t="n"/>
       <c r="F26" s="11">
@@ -3957,16 +4077,16 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Tuerca M8</t>
+          <t>Tornillo M3 x 8 + inserto termico M3 (bandejas)</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="11">
@@ -3982,16 +4102,16 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Arandela ancha DIN 9021</t>
+          <t>Tornillo M3 x 16 + tuerca (capsulas)</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E28" s="12" t="n"/>
       <c r="F28" s="11">
@@ -4007,16 +4127,16 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M4 x 14 + tuerca (uniones de tramos)</t>
+          <t>Tornillo M2 autorroscante (bisel)</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2 x 6</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E29" s="12" t="n"/>
       <c r="F29" s="11">
@@ -4032,16 +4152,16 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Tornillo M3 x 8 avellanado + inserto M3 (tapa del bolsillo)</t>
+          <t>Cordon de junta torica Ø2 (caja + 2 capsulas, +10 %)</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>970 mm</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E30" s="12" t="n"/>
       <c r="F30" s="11">
@@ -4057,16 +4177,16 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Perno M4 hexagonal (perillas) + tuerca en la ranura T</t>
+          <t>Prensaestopas PG7 con contratuerca (3 caja + 2 capsulas)</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>PG7</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="11">
@@ -4082,12 +4202,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Perno M4 x 20 + tuerca mariposa (bisagras)</t>
+          <t>Disco de acrilico de la ventana</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>Ø30 x 3</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
@@ -4107,16 +4227,16 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Pivote M3 del pestillo</t>
+          <t>Grillete o argolla de inox (izado)</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="D33" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="12" t="n"/>
       <c r="F33" s="11">
@@ -4132,16 +4252,16 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Correa textil</t>
+          <t>Tornillo M4 x 12 + inserto termico M4 (riel a la caja)</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>25 x 300 mm</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="D34" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E34" s="12" t="n"/>
       <c r="F34" s="11">
@@ -4157,20 +4277,245 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Pletina de inox</t>
+          <t>Varilla roscada M8 (8.8)</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>25 x 5 x 100</t>
+          <t>451 mm</t>
         </is>
       </c>
       <c r="D35" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E35" s="12" t="n"/>
       <c r="F35" s="11">
         <f>D35*E35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Tuerca M8</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="11">
+        <f>D36*E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Arandela ancha DIN 9021</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="11">
+        <f>D37*E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Tornillo M4 x 14 + tuerca (uniones de tramos)</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="11">
+        <f>D38*E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Tornillo M3 x 8 avellanado + inserto M3 (tapa del bolsillo)</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="11">
+        <f>D39*E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Perno M4 hexagonal (perillas) + tuerca en la ranura T</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="11">
+        <f>D40*E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Perno M4 x 20 + tuerca mariposa (bisagras)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="11">
+        <f>D41*E41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Pivote M3 del pestillo</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="11">
+        <f>D42*E42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Correa textil</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>25 x 300 mm</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="11">
+        <f>D43*E43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>modular D200</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Pletina de inox</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>25 x 5 x 100</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="11">
+        <f>D44*E44</f>
         <v/>
       </c>
     </row>
@@ -4185,13 +4530,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4219,11 +4564,13 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Riel: largo</t>
-        </is>
-      </c>
-      <c r="B2" s="11" t="n">
-        <v>430</v>
+          <t>Riel: largo / seccion x pared</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>430 / 30 x 4</t>
+        </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4232,29 +4579,29 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>params.py simple.riel_L</t>
+          <t>params.py simple.riel_L, riel.*</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Riel: seccion x pared</t>
+          <t>Caja: ESP32 y pisos</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>30 x 4</t>
+          <t>kit_a, 2 pisos</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>params.py riel.seccion, riel.pared</t>
+          <t>params.py simple.esp32_base (equipo), simple.caja_pisos</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4613,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>139.6 x 106.0 x 50.0</t>
+          <t>127.0 x 126.0 x 77.0</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -4288,7 +4635,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>159.6 x 126.0</t>
+          <t>147.0 x 146.0</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -4310,7 +4657,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>131.6 x 98.0 x 46.0</t>
+          <t>119.0 x 118.0 x 73.0</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -4349,12 +4696,12 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Capsula: exterior (largo x ancho x alto)</t>
+          <t>Nodo sobre el aro (de / a)</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>44.0 x 46.0 x 46.0</t>
+          <t>-40 / 181</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -4364,19 +4711,19 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>capsula.py cap_dims</t>
+          <t>simple.py, nube de puntos del CAD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Capsula: cavidad</t>
+          <t>Capsula: exterior</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>38.0 x 38.0 x 38.0</t>
+          <t>44.0 x 46.0 x 46.0</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -4386,27 +4733,29 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>capsula.py (camara + holguras)</t>
+          <t>capsula.py cap_dims</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Capsula: angulo fijo</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="n">
-        <v>30</v>
+          <t>Capsula: angulo y acimut</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>30 grados, adentro</t>
+        </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>grados</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>params.py capsula.angulo</t>
+          <t>params.py capsula.angulo, capsula.acimut (equipo)</t>
         </is>
       </c>
     </row>
@@ -4433,9 +4782,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Gancho: C interior / pared / asiento</t>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Gancho en C (fusionado al riel): C interior / pared / asiento</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -4457,11 +4806,13 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Gancho: fondo del riel al centro de la varilla</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>40</v>
+          <t>Separador LR1: tipo, seccion, altura (minima)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>aro, 12 x 6, 140 (136)</t>
+        </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
@@ -4470,19 +4821,19 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>params.py gancho.caida</t>
+          <t>params.py separador.*, simple.py</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Separador LR1: tipo, seccion</t>
+          <t>Pletinas de lastre</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>aro, 12 x 6</t>
+          <t>5 x 2 de 25 x 5 x 100</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -4492,107 +4843,107 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>params.py separador.*</t>
+          <t>params.py lastre.pletinas</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Separador: altura (minima calculada)</t>
+          <t>Nodo: peso en aire (bandeja 40 % / 100 %)</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>250 (165)</t>
+          <t>2450 / 2458</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>g</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>simple.py min_separator_h</t>
+          <t>simple.py, masas por pieza con su relleno</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Pletinas de lastre</t>
+          <t>Nodo: peso aparente (40 % / 100 %)</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>3 x 2 de 25 x 5 x 100</t>
+          <t>+203 / +211</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>g</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>params.py lastre.pletinas</t>
+          <t>simple.py (ventana +200 a +500)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Peso en aire (bandeja 40 % / 100 %)</t>
+          <t>Nodo: BG</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>2079 / 2083</t>
+          <t>18.3</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>simple.py, volumenes del CAD</t>
+          <t>simple.py</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Peso aparente en el agua (40 % / 100 %)</t>
+          <t>Apice sobre el aro</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>+265 / +269</t>
+          <t>290</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>simple.py (ventana +200 a +500)</t>
+          <t>separador.altura + apice.altura</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Estabilidad BG</t>
+          <t>Aire minimo suspension-nodo</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -4602,63 +4953,63 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>simple.py centros de masa y empuje</t>
+          <t>simple.py (exigido 10)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Apice sobre el aro</t>
+          <t>FS riel (capas / entre capas)</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>19.3 / 9.4</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>separador.altura + apice.altura</t>
+          <t>simple.py §5, a mano</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Aire minimo suspension-nodo</t>
+          <t>FS pie de capsula (capas / entre capas)</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>4.2 / 2.1</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>simple.py, nube de puntos del CAD (exigido 10)</t>
+          <t>simple.py §5, a mano</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>FS del riel (a lo largo / entre capas)</t>
+          <t>FS gancho (capas / entre capas)</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>6.9 / 3.4</t>
+          <t>6.0 / 2.9</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -4668,73 +5019,161 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>simple.py §5</t>
+          <t>simple.py §5, a mano</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>FS del pie de capsula (a lo largo / entre capas)</t>
+          <t>Traccion por inserto M4 de las bridas al izar</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>2.5 / 1.2</t>
+          <t>324</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>simple.py §5 (punto debil)</t>
+          <t>simple.py §5 (probar con PB8)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Traccion por inserto M4 al izar</t>
+          <t>Cable por camara</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>381</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>simple.py §5</t>
+          <t>simple.py §6 (&gt; 300: prueba SPI)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Cable por camara</t>
+          <t>Boya: masa / calado / francobordo</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>2705 / 31.6 / 88.4</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
+          <t>g / mm / mm</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>boya_simple.py (agua de mar 1025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Boya: reserva / GM balanceo y cabeceo</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>194 % / 92 y 467</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>- / mm</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>boya_simple.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Nodo + boya en aire (limite 3000)</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>5155</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>simple.py + boya_simple.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Camara en Ø200: lente a la red</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>simple.py §6 (&gt; 300: prueba SPI)</t>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>simple.py camera_view (FOV y enfoque estimados)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Camara en Ø500: lente a la red</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>no corta la red</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>simple.py camera_view (FOV y enfoque estimados)</t>
         </is>
       </c>
     </row>
@@ -6687,7 +7126,7 @@
       </c>
       <c r="J42" s="11" t="inlineStr">
         <is>
-          <t>umbilical[1]</t>
+          <t>umbilical.longitud</t>
         </is>
       </c>
       <c r="K42" s="11" t="inlineStr"/>

</xml_diff>

<commit_message>
cad(bloqueF): bitacora con P2, P4 y la boya PET 4 x 1 L
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Proyecto/MóduloMecánico/salida/simple/BITACORA.xlsx
+++ b/Proyecto/MóduloMecánico/salida/simple/BITACORA.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -751,16 +751,105 @@
       <c r="F15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A16,PIEZAS!$N:$N)</f>
+        <v/>
+      </c>
+      <c r="C16" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A16,PIEZAS!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="D16" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A16,PIEZAS!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="E16" s="2">
+        <f>SUMIF(HARDWARE!$A:$A,$A16,HARDWARE!$F:$F)</f>
+        <v/>
+      </c>
+      <c r="F16" s="2">
+        <f>D16+E16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A17,PIEZAS!$N:$N)</f>
+        <v/>
+      </c>
+      <c r="C17" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A17,PIEZAS!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="D17" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A17,PIEZAS!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="E17" s="2">
+        <f>SUMIF(HARDWARE!$A:$A,$A17,HARDWARE!$F:$F)</f>
+        <v/>
+      </c>
+      <c r="F17" s="2">
+        <f>D17+E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A18,PIEZAS!$N:$N)</f>
+        <v/>
+      </c>
+      <c r="C18" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A18,PIEZAS!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="D18" s="2">
+        <f>SUMIF(PIEZAS!$B:$B,$A18,PIEZAS!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="E18" s="2">
+        <f>SUMIF(HARDWARE!$A:$A,$A18,HARDWARE!$F:$F)</f>
+        <v/>
+      </c>
+      <c r="F18" s="2">
+        <f>D18+E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Masa por pieza = la misma del calculo de flotacion (piel + relleno de cada pieza). Llenar los precios amarillos de HARDWARE para el costo total. La fila modular D200 es para comparar.</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -773,11 +862,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R34"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
@@ -914,14 +1003,14 @@
         <v>146</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>102.5</v>
+        <v>107</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>349.39</v>
+        <v>383.45</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1130,13 +1219,13 @@
         <v>117</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>11.14</v>
+        <v>19.91</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -1548,61 +1637,63 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>LR1_separador</t>
+          <t>B1s_casco</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>linterna de prueba</t>
+          <t>boya simple</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>LR1 separador</t>
+          <t>B1s casco</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>211.9</v>
+        <v>240</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>211.9</v>
+        <v>220</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>44.86</v>
+        <v>753.49</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0.766</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>37</v>
+        <v>1</v>
+      </c>
+      <c r="M11" s="2">
+        <f>H11*RESUMEN!$B$3*L11</f>
+        <v/>
       </c>
       <c r="N11" s="2">
         <f>M11*D11</f>
         <v/>
       </c>
-      <c r="O11" s="2" t="n">
-        <v>1.56</v>
+      <c r="O11" s="2">
+        <f>M11/RESUMEN!$B$4</f>
+        <v/>
       </c>
       <c r="P11" s="2">
         <f>O11*D11</f>
@@ -1614,14 +1705,14 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>slicer</t>
+          <t>estimado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>B1s_casco</t>
+          <t>B2s_tapa</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1631,27 +1722,27 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>B1s casco</t>
+          <t>B2s tapa</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>240</v>
+        <v>9</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>220</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>125</v>
+        <v>240</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>753.49</v>
+        <v>260.46</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1696,7 +1787,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>B2s_tapa</t>
+          <t>B1bs_bandeja</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1706,41 +1797,41 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>B2s tapa</t>
+          <t>B1bs bandeja</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>9</v>
+        <v>206</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>220</v>
+        <v>186</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>240</v>
+        <v>3</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>260.46</v>
+        <v>112.95</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>100 %</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="L13" s="2" t="n">
-        <v>1</v>
+        <v>0.897</v>
       </c>
       <c r="M13" s="2">
         <f>H13*RESUMEN!$B$3*L13</f>
@@ -1771,7 +1862,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>B1bs_bandeja</t>
+          <t>B3s_larguero</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1781,27 +1872,27 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>B1bs bandeja</t>
+          <t>B3s larguero del panel</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>206</v>
+        <v>24</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>112.95</v>
+        <v>28.42</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1815,7 +1906,7 @@
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>0.897</v>
+        <v>0.714</v>
       </c>
       <c r="M14" s="2">
         <f>H14*RESUMEN!$B$3*L14</f>
@@ -1846,7 +1937,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>B3s_larguero</t>
+          <t>B5s_flotador</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1856,41 +1947,41 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>B3s larguero del panel</t>
+          <t>B5s flotador de esquina</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>28.42</v>
+        <v>91.47</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0.714</v>
+        <v>1</v>
       </c>
       <c r="M15" s="2">
         <f>H15*RESUMEN!$B$3*L15</f>
@@ -1921,7 +2012,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>B5s_flotador</t>
+          <t>B6s_ojal</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1931,32 +2022,32 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>B5s flotador de esquina</t>
+          <t>B6s ojal de amarre</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>91.47</v>
+        <v>8.31</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1996,42 +2087,42 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>B6s_ojal</t>
+          <t>M1_caja_cuerpo</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>boya simple</t>
+          <t>modular D200</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>B6s ojal de amarre</t>
+          <t>Caja, cuerpo</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>30</v>
+        <v>159.6</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>8.31</v>
+        <v>214.82</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2071,7 +2162,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>M1_caja_cuerpo</t>
+          <t>M2_caja_tapa</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2081,27 +2172,27 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Caja, cuerpo</t>
+          <t>Caja, tapa con asa</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>159.6</v>
+        <v>63</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>126</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>50</v>
+        <v>159.6</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>214.82</v>
+        <v>129.41</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2146,7 +2237,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>M2_caja_tapa</t>
+          <t>M11_bandeja</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -2156,41 +2247,41 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Caja, tapa con asa</t>
+          <t>Bandeja</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>63</v>
+        <v>127.6</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>126</v>
+        <v>94</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>159.6</v>
+        <v>18</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>129.41</v>
+        <v>35.64</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>sin girar</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>100 %</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="L19" s="2" t="n">
-        <v>1</v>
+        <v>0.912</v>
       </c>
       <c r="M19" s="2">
         <f>H19*RESUMEN!$B$3*L19</f>
@@ -2221,7 +2312,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>M11_bandeja</t>
+          <t>M3_riel_central</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2231,41 +2322,41 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Bandeja</t>
+          <t>Riel, tramo central</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>127.6</v>
+        <v>69.8</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>35.64</v>
+        <v>170.11</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>sin girar</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0.912</v>
+        <v>1</v>
       </c>
       <c r="M20" s="2">
         <f>H20*RESUMEN!$B$3*L20</f>
@@ -2296,7 +2387,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>M3_riel_central</t>
+          <t>M3_riel_ext</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2306,23 +2397,23 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Riel, tramo central</t>
+          <t>Riel, extension</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>69.8</v>
+        <v>30</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>170.11</v>
+        <v>44.76</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
@@ -2371,7 +2462,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>M3_riel_ext</t>
+          <t>M3_riel_punta</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2381,7 +2472,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Riel, extension</t>
+          <t>Riel, punta</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -2394,10 +2485,10 @@
         <v>30</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>44.76</v>
+        <v>25.32</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -2411,11 +2502,11 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>100 %</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="L22" s="2" t="n">
-        <v>1</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="M22" s="2">
         <f>H22*RESUMEN!$B$3*L22</f>
@@ -2446,7 +2537,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>M3_riel_punta</t>
+          <t>M3_tapa_bolsillo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2456,32 +2547,32 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Riel, punta</t>
+          <t>Tapa del bolsillo</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>30</v>
+        <v>107</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>25.32</v>
+        <v>9.58</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2490,7 +2581,7 @@
         </is>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.953</v>
       </c>
       <c r="M23" s="2">
         <f>H23*RESUMEN!$B$3*L23</f>
@@ -2521,7 +2612,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>M3_tapa_bolsillo</t>
+          <t>M4_capsula_cuerpo</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2531,41 +2622,41 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Tapa del bolsillo</t>
+          <t>Capsula, cuerpo</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>9.58</v>
+        <v>45.95</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>Y-90</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0.953</v>
+        <v>1</v>
       </c>
       <c r="M24" s="2">
         <f>H24*RESUMEN!$B$3*L24</f>
@@ -2596,7 +2687,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>M4_capsula_cuerpo</t>
+          <t>M5_capsula_tapa</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2606,27 +2697,27 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Capsula, cuerpo</t>
+          <t>Capsula, tapa con bisagra</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>64</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>45.95</v>
+        <v>23.47</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Y-90</t>
+          <t>X-90</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2671,7 +2762,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>M5_capsula_tapa</t>
+          <t>M6_capsula_bisel</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2681,37 +2772,37 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Capsula, tapa con bisagra</t>
+          <t>Bisel</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>64</v>
+        <v>2.5</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>23.47</v>
+        <v>1.89</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>X-90</t>
+          <t>Y+90</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>100 %</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="L26" s="2" t="n">
@@ -2746,7 +2837,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>M6_capsula_bisel</t>
+          <t>M9_gancho</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2756,23 +2847,23 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Bisel</t>
+          <t>Gancho al aro</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2.5</v>
+        <v>68</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>1.89</v>
+        <v>19.51</v>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
@@ -2781,7 +2872,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2790,7 +2881,7 @@
         </is>
       </c>
       <c r="L27" s="2" t="n">
-        <v>1</v>
+        <v>0.735</v>
       </c>
       <c r="M27" s="2">
         <f>H27*RESUMEN!$B$3*L27</f>
@@ -2821,7 +2912,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>M9_gancho</t>
+          <t>M10_carro_capsula</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2831,27 +2922,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Gancho al aro</t>
+          <t>Carro</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>59</v>
+        <v>80.8</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>30</v>
+        <v>38.6</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>19.51</v>
+        <v>54.5</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Y+90</t>
+          <t>Y-90</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2865,7 +2956,7 @@
         </is>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0.735</v>
+        <v>0.71</v>
       </c>
       <c r="M28" s="2">
         <f>H28*RESUMEN!$B$3*L28</f>
@@ -2896,7 +2987,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>M10_carro_capsula</t>
+          <t>M12_perilla</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2906,32 +2997,32 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Carro</t>
+          <t>Perilla</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>80.8</v>
+        <v>30</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>38.6</v>
+        <v>30</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>54.5</v>
+        <v>6.71</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Y-90</t>
+          <t>X180</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2940,7 +3031,7 @@
         </is>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0.71</v>
+        <v>0.695</v>
       </c>
       <c r="M29" s="2">
         <f>H29*RESUMEN!$B$3*L29</f>
@@ -2971,7 +3062,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>M12_perilla</t>
+          <t>M13_casquillo_D8</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2981,27 +3072,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Perilla</t>
+          <t>Casquillo Ø8</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>30</v>
+        <v>15.7</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>6.71</v>
+        <v>1.61</v>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>X180</t>
+          <t>X-90</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3015,7 +3106,7 @@
         </is>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0.695</v>
+        <v>0.972</v>
       </c>
       <c r="M30" s="2">
         <f>H30*RESUMEN!$B$3*L30</f>
@@ -3046,7 +3137,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>M13_casquillo_D8</t>
+          <t>M14_pestillo</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -3056,27 +3147,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Casquillo Ø8</t>
+          <t>Pestillo</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>15.7</v>
+        <v>12</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>20</v>
+        <v>35.2</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>13.5</v>
+        <v>3.6</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>1.61</v>
+        <v>0.92</v>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>X-90</t>
+          <t>X+90</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -3090,7 +3181,7 @@
         </is>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0.972</v>
+        <v>1</v>
       </c>
       <c r="M31" s="2">
         <f>H31*RESUMEN!$B$3*L31</f>
@@ -3121,63 +3212,61 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>M14_pestillo</t>
+          <t>M1s_caja_cuerpo</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>modular D200</t>
+          <t>nodo P2 robusto</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Pestillo</t>
+          <t>M1s_caja_cuerpo</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>35.2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>X+90</t>
+          <t>slicer</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>100 %</t>
         </is>
       </c>
       <c r="L32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M32" s="2">
-        <f>H32*RESUMEN!$B$3*L32</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>509.2</v>
       </c>
       <c r="N32" s="2">
         <f>M32*D32</f>
         <v/>
       </c>
-      <c r="O32" s="2">
-        <f>M32/RESUMEN!$B$4</f>
-        <v/>
+      <c r="O32" s="2" t="n">
+        <v>16.13</v>
       </c>
       <c r="P32" s="2">
         <f>O32*D32</f>
@@ -3189,53 +3278,1732 @@
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>estimado</t>
+          <t>slicer</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="n"/>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="n"/>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>M2_caja_tapa</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>M2_caja_tapa</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>181.2</v>
+      </c>
+      <c r="N33" s="2">
+        <f>M33*D33</f>
+        <v/>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="P33" s="2">
+        <f>O33*D33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="2">
+        <f>N33/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>M3s_riel_gancho</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>M3s_riel_gancho</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>137.1</v>
+      </c>
+      <c r="N34" s="2">
+        <f>M34*D34</f>
+        <v/>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="P34" s="2">
+        <f>O34*D34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="2">
+        <f>N34/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>M3t_tapa_bolsillo</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>M3t_tapa_bolsillo</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="N35" s="2">
+        <f>M35*D35</f>
+        <v/>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="P35" s="2">
+        <f>O35*D35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="2">
+        <f>N35/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>M5s_capsula_tapa_pie</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>M5s_capsula_tapa_pie</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="N36" s="2">
+        <f>M36*D36</f>
+        <v/>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="P36" s="2">
+        <f>O36*D36</f>
+        <v/>
+      </c>
+      <c r="Q36" s="2">
+        <f>N36/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="N37" s="2">
+        <f>M37*D37</f>
+        <v/>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="P37" s="2">
+        <f>O37*D37</f>
+        <v/>
+      </c>
+      <c r="Q37" s="2">
+        <f>N37/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja_sup</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja_sup</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="N38" s="2">
+        <f>M38*D38</f>
+        <v/>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="P38" s="2">
+        <f>O38*D38</f>
+        <v/>
+      </c>
+      <c r="Q38" s="2">
+        <f>N38/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>M4_capsula_cuerpo</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>M4_capsula_cuerpo</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="N39" s="2">
+        <f>M39*D39</f>
+        <v/>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P39" s="2">
+        <f>O39*D39</f>
+        <v/>
+      </c>
+      <c r="Q39" s="2">
+        <f>N39/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>M6_capsula_bisel</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>nodo P2 robusto</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>M6_capsula_bisel</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N40" s="2">
+        <f>M40*D40</f>
+        <v/>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P40" s="2">
+        <f>O40*D40</f>
+        <v/>
+      </c>
+      <c r="Q40" s="2">
+        <f>N40/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>M1m_caja_riel</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>M1m_caja_riel</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>675.3</v>
+      </c>
+      <c r="N41" s="2">
+        <f>M41*D41</f>
+        <v/>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="P41" s="2">
+        <f>O41*D41</f>
+        <v/>
+      </c>
+      <c r="Q41" s="2">
+        <f>N41/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>M2_caja_tapa</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>M2_caja_tapa</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>170.7</v>
+      </c>
+      <c r="N42" s="2">
+        <f>M42*D42</f>
+        <v/>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="P42" s="2">
+        <f>O42*D42</f>
+        <v/>
+      </c>
+      <c r="Q42" s="2">
+        <f>N42/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>M3t_tapa_bolsillo</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>M3t_tapa_bolsillo</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="N43" s="2">
+        <f>M43*D43</f>
+        <v/>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="P43" s="2">
+        <f>O43*D43</f>
+        <v/>
+      </c>
+      <c r="Q43" s="2">
+        <f>N43/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>M5m_extremo_pie</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>M5m_extremo_pie</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="N44" s="2">
+        <f>M44*D44</f>
+        <v/>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="P44" s="2">
+        <f>O44*D44</f>
+        <v/>
+      </c>
+      <c r="Q44" s="2">
+        <f>N44/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>M9c_abrazadera</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>M9c_abrazadera</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="N45" s="2">
+        <f>M45*D45</f>
+        <v/>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="P45" s="2">
+        <f>O45*D45</f>
+        <v/>
+      </c>
+      <c r="Q45" s="2">
+        <f>N45/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="N46" s="2">
+        <f>M46*D46</f>
+        <v/>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="P46" s="2">
+        <f>O46*D46</f>
+        <v/>
+      </c>
+      <c r="Q46" s="2">
+        <f>N46/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja_sup</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>M11_bandeja_sup</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="N47" s="2">
+        <f>M47*D47</f>
+        <v/>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="P47" s="2">
+        <f>O47*D47</f>
+        <v/>
+      </c>
+      <c r="Q47" s="2">
+        <f>N47/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>M4_capsula_cuerpo</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>M4_capsula_cuerpo</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="2" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="N48" s="2">
+        <f>M48*D48</f>
+        <v/>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P48" s="2">
+        <f>O48*D48</f>
+        <v/>
+      </c>
+      <c r="Q48" s="2">
+        <f>N48/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>M6_capsula_bisel</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>nodo P4 estetico</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>M6_capsula_bisel</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N49" s="2">
+        <f>M49*D49</f>
+        <v/>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P49" s="2">
+        <f>O49*D49</f>
+        <v/>
+      </c>
+      <c r="Q49" s="2">
+        <f>N49/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>B1_casco</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>B1 casco</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>213.6</v>
+      </c>
+      <c r="N50" s="2">
+        <f>M50*D50</f>
+        <v/>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="P50" s="2">
+        <f>O50*D50</f>
+        <v/>
+      </c>
+      <c r="Q50" s="2">
+        <f>N50/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>B2_cubierta</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>B2 cubierta</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="N51" s="2">
+        <f>M51*D51</f>
+        <v/>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P51" s="2">
+        <f>O51*D51</f>
+        <v/>
+      </c>
+      <c r="Q51" s="2">
+        <f>N51/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>B3_caja</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>B3 caja seca</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="N52" s="2">
+        <f>M52*D52</f>
+        <v/>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="P52" s="2">
+        <f>O52*D52</f>
+        <v/>
+      </c>
+      <c r="Q52" s="2">
+        <f>N52/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>B4_tapa</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>B4 tapa</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="2" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="N53" s="2">
+        <f>M53*D53</f>
+        <v/>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="P53" s="2">
+        <f>O53*D53</f>
+        <v/>
+      </c>
+      <c r="Q53" s="2">
+        <f>N53/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>B5_cuna</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>B5 cuna</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="N54" s="2">
+        <f>M54*D54</f>
+        <v/>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="P54" s="2">
+        <f>O54*D54</f>
+        <v/>
+      </c>
+      <c r="Q54" s="2">
+        <f>N54/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>B6_correa</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>boya PET 4 x 1 L</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>B6 correa</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="N55" s="2">
+        <f>M55*D55</f>
+        <v/>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P55" s="2">
+        <f>O55*D55</f>
+        <v/>
+      </c>
+      <c r="Q55" s="2">
+        <f>N55/1000*RESUMEN!$B$5</f>
+        <v/>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>slicer</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="n"/>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="n"/>
+      <c r="P56" s="2" t="n"/>
+      <c r="Q56" s="2" t="n"/>
+      <c r="R56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Soportes: voladizo en la orientacion de impresion &gt; 300 mm². Masa = volumen x densidad x fraccion maciza (piel de impresion.cascara + relleno); horas = masa / g por hora (RESUMEN).</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="n"/>
+      <c r="N57" s="2" t="n"/>
+      <c r="O57" s="2" t="n"/>
+      <c r="P57" s="2" t="n"/>
+      <c r="Q57" s="2" t="n"/>
+      <c r="R57" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3599,16 +5367,16 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Pletina de inox</t>
+          <t>Lastre a granel: tuercas y arandelas M8 de inox</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>25 x 5 x 100</t>
+          <t>1140 g</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="2">
@@ -4381,7 +6149,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="57" customWidth="1" min="4" max="4"/>
   </cols>
@@ -4653,34 +6421,34 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Separador LR1: tipo, seccion, altura (minima)</t>
+          <t>Separador LR1</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>aro, 12 x 6, 140 (136)</t>
+          <t>no se usa</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>params.py separador.*, simple.py</t>
+          <t>params.py separador.usar (tanda 3: sin separador)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Pletinas de lastre</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>5 x 2 de 25 x 5 x 100</t>
+          <t>Lastre a granel (un bolsillo por lado)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>1140 g de tuercas y arandelas M8 de inox, a granel, bolsillo 100 x 50 x 30</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -4690,7 +6458,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>params.py lastre.pletinas</t>
+          <t>params.py lastre.granel, simple.py</t>
         </is>
       </c>
     </row>
@@ -4702,7 +6470,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2462 / 2471</t>
+          <t>2680 / 2689</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -4724,7 +6492,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+205 / +214</t>
+          <t>+350 / +359</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4746,7 +6514,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>18.2</t>
+          <t>20.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -4763,12 +6531,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Apice sobre el aro</t>
+          <t>Punto de amarre de las cuerdas sobre el aro</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>400</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -4778,7 +6546,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>separador.altura + apice.altura</t>
+          <t>linterna.nudo_h</t>
         </is>
       </c>
     </row>
@@ -4790,7 +6558,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">

</xml_diff>